<commit_message>
📦Abgabebereit  (Messdaten validiert mit Sim)
</commit_message>
<xml_diff>
--- a/EX01/Oszi6-R_S-L_S.xlsx
+++ b/EX01/Oszi6-R_S-L_S.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paulkronegger/Library/CloudStorage/SynologyDrive-mbp-paul/Segeln/Trainer/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos-jku\EMTS-PR\EX01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752CB613-3A32-FD4C-9D1F-567B663FD856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602586D1-FF3C-4E59-8519-3A72A8F6C9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{C0B4212B-C46B-1042-A4F8-FD95F2F6CE51}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C0B4212B-C46B-1042-A4F8-FD95F2F6CE51}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,6 +27,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -66,7 +67,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -99,7 +100,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -212,9 +213,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -252,7 +253,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -358,7 +359,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -500,7 +501,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -509,13 +510,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7C84A01-45A9-284D-BB97-8281FC50E5D9}">
   <dimension ref="A1:I4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="12.625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -541,91 +542,91 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>3.6</v>
+        <v>1.2</v>
       </c>
       <c r="B2">
         <v>50</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="D2">
-        <v>15</v>
+        <v>19.8</v>
       </c>
       <c r="E2">
         <v>50</v>
       </c>
       <c r="G2" s="2">
         <f>A2*B2/C2*COS(D2/180*PI())</f>
-        <v>43.466662183008076</v>
+        <v>14.856012141382509</v>
       </c>
       <c r="H2" s="1">
         <f>A2*B2/C2*SIN(D2/180*PI())</f>
-        <v>11.646857029613432</v>
+        <v>5.3484934775572324</v>
       </c>
       <c r="I2" s="1">
         <f>H2/(2*PI()*E2)</f>
-        <v>3.7073097354951338E-2</v>
+        <v>1.7024783500959893E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>3.9</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="B3">
         <v>50</v>
       </c>
       <c r="C3">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
       <c r="D3">
-        <v>60</v>
+        <v>61.2</v>
       </c>
       <c r="E3">
         <v>50</v>
       </c>
       <c r="G3" s="2">
         <f t="shared" ref="G3:G4" si="0">A3*B3/C3*COS(D3/180*PI())</f>
-        <v>26.351351351351358</v>
+        <v>15.140829757482479</v>
       </c>
       <c r="H3" s="1">
         <f t="shared" ref="H3:H4" si="1">A3*B3/C3*SIN(D3/180*PI())</f>
-        <v>45.641879388639332</v>
+        <v>27.541067087092863</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" ref="I3:I4" si="2">H3/(2*PI()*E3)</f>
-        <v>0.14528261433412087</v>
+        <v>8.7665939298726722E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4">
-        <v>0.52</v>
+        <v>0.32</v>
       </c>
       <c r="D4">
-        <v>65</v>
+        <v>88.2</v>
       </c>
       <c r="E4">
         <v>50</v>
       </c>
       <c r="G4" s="2">
         <f t="shared" si="0"/>
-        <v>365.72734189098986</v>
+        <v>24.048862419192055</v>
       </c>
       <c r="H4" s="1">
         <f t="shared" si="1"/>
-        <v>784.30481570479321</v>
+        <v>765.24721028001341</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" si="2"/>
-        <v>2.4965197662039165</v>
+        <v>2.435857524066944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>